<commit_message>
Publish Copenhagen_2013_MAR, Duisburg_2013_WCH, Racice_2013_WC, Welland_2013_JWCH
</commit_message>
<xml_diff>
--- a/events/Copenhagen_2013_MAR/Copenhagen_2013_MAR_Results.xlsx
+++ b/events/Copenhagen_2013_MAR/Copenhagen_2013_MAR_Results.xlsx
@@ -22621,6 +22621,11 @@
           <t>02:13:09.000</t>
         </is>
       </c>
+      <c r="R338" t="inlineStr">
+        <is>
+          <t>161210</t>
+        </is>
+      </c>
     </row>
     <row r="339">
       <c r="A339" t="inlineStr">
@@ -23466,7 +23471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D234"/>
+  <dimension ref="A1:D235"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -28617,6 +28622,28 @@
         </is>
       </c>
     </row>
+    <row r="235">
+      <c r="A235" t="inlineStr">
+        <is>
+          <t>161210</t>
+        </is>
+      </c>
+      <c r="B235" t="inlineStr">
+        <is>
+          <t>Gaston</t>
+        </is>
+      </c>
+      <c r="C235" t="inlineStr">
+        <is>
+          <t>GAONA</t>
+        </is>
+      </c>
+      <c r="D235" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>